<commit_message>
Sprint 5 Day 32: Add capital allocation analysis
</commit_message>
<xml_diff>
--- a/output/cashflow_intelligence.xlsx
+++ b/output/cashflow_intelligence.xlsx
@@ -9,6 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cashflow_intelligence" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="allocation_distribution" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="allocation_changes" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -426,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K93"/>
+  <dimension ref="A1:M93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -485,6 +487,16 @@
           <t>capital_allocation_label</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>latest_capital_allocation</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>capital_allocation_year</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -528,6 +540,14 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -571,6 +591,14 @@
           <t>Mixed</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -616,6 +644,14 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -660,6 +696,14 @@
         <is>
           <t>Liquidating Assets</t>
         </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>2024</v>
       </c>
     </row>
     <row r="6">
@@ -704,6 +748,14 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -749,6 +801,14 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -794,6 +854,14 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -839,6 +907,14 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -883,6 +959,14 @@
         <is>
           <t>Reinvestor</t>
         </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>2024</v>
       </c>
     </row>
     <row r="11">
@@ -927,6 +1011,14 @@
           <t>Growth Funded by Debt</t>
         </is>
       </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -972,6 +1064,14 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M12" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1016,6 +1116,14 @@
         <is>
           <t>Mixed</t>
         </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="M13" t="n">
+        <v>2024</v>
       </c>
     </row>
     <row r="14">
@@ -1060,6 +1168,14 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M14" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1104,6 +1220,14 @@
         <is>
           <t>Reinvestor</t>
         </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M15" t="n">
+        <v>2024</v>
       </c>
     </row>
     <row r="16">
@@ -1148,6 +1272,14 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M16" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1191,6 +1323,14 @@
           <t>Growth Funded by Debt</t>
         </is>
       </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="M17" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1236,6 +1376,14 @@
           <t>Liquidating Assets</t>
         </is>
       </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="M18" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1280,6 +1428,14 @@
         <is>
           <t>Shareholder Returns</t>
         </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M19" t="n">
+        <v>2024</v>
       </c>
     </row>
     <row r="20">
@@ -1324,6 +1480,14 @@
           <t>Mixed</t>
         </is>
       </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="M20" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1369,6 +1533,14 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M21" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1414,6 +1586,14 @@
           <t>Liquidating Assets</t>
         </is>
       </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="M22" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1459,6 +1639,14 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M23" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1503,6 +1691,14 @@
         <is>
           <t>Mixed</t>
         </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="M24" t="n">
+        <v>2024</v>
       </c>
     </row>
     <row r="25">
@@ -1547,6 +1743,14 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M25" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1590,6 +1794,14 @@
           <t>Mixed</t>
         </is>
       </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="M26" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1635,6 +1847,14 @@
           <t>Liquidating Assets</t>
         </is>
       </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="M27" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1679,6 +1899,14 @@
         <is>
           <t>Shareholder Returns</t>
         </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M28" t="n">
+        <v>2024</v>
       </c>
     </row>
     <row r="29">
@@ -1723,6 +1951,14 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M29" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1767,6 +2003,14 @@
         <is>
           <t>Shareholder Returns</t>
         </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M30" t="n">
+        <v>2024</v>
       </c>
     </row>
     <row r="31">
@@ -1811,6 +2055,14 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M31" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1854,6 +2106,14 @@
           <t>Mixed</t>
         </is>
       </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="M32" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1898,6 +2158,14 @@
         <is>
           <t>Shareholder Returns</t>
         </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M33" t="n">
+        <v>2024</v>
       </c>
     </row>
     <row r="34">
@@ -1942,6 +2210,14 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M34" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1987,6 +2263,14 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M35" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2031,6 +2315,14 @@
         <is>
           <t>Shareholder Returns</t>
         </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M36" t="n">
+        <v>2024</v>
       </c>
     </row>
     <row r="37">
@@ -2075,6 +2367,14 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M37" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2119,6 +2419,14 @@
         <is>
           <t>Shareholder Returns</t>
         </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M38" t="n">
+        <v>2024</v>
       </c>
     </row>
     <row r="39">
@@ -2163,6 +2471,14 @@
           <t>Growth Funded by Debt</t>
         </is>
       </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="M39" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2206,6 +2522,14 @@
           <t>Growth Funded by Debt</t>
         </is>
       </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="M40" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2250,6 +2574,14 @@
         <is>
           <t>Reinvestor</t>
         </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M41" t="n">
+        <v>2024</v>
       </c>
     </row>
     <row r="42">
@@ -2294,6 +2626,14 @@
           <t>Growth Funded by Debt</t>
         </is>
       </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="M42" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2337,6 +2677,14 @@
           <t>Growth Funded by Debt</t>
         </is>
       </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="M43" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2381,6 +2729,14 @@
         <is>
           <t>Reinvestor</t>
         </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M44" t="n">
+        <v>2024</v>
       </c>
     </row>
     <row r="45">
@@ -2425,6 +2781,14 @@
           <t>Growth Funded by Debt</t>
         </is>
       </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="M45" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2468,6 +2832,14 @@
           <t>Liquidating Assets</t>
         </is>
       </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="M46" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2511,6 +2883,14 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M47" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2556,6 +2936,14 @@
           <t>Mixed</t>
         </is>
       </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="M48" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2601,6 +2989,14 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M49" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2645,6 +3041,14 @@
         <is>
           <t>Mixed</t>
         </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="M50" t="n">
+        <v>2024</v>
       </c>
     </row>
     <row r="51">
@@ -2689,6 +3093,14 @@
           <t>Pre-Revenue</t>
         </is>
       </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>Pre-Revenue</t>
+        </is>
+      </c>
+      <c r="M51" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2732,6 +3144,14 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M52" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2775,6 +3195,14 @@
           <t>Mixed</t>
         </is>
       </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="M53" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2818,6 +3246,14 @@
           <t>Mixed</t>
         </is>
       </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="M54" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2862,6 +3298,14 @@
         <is>
           <t>Reinvestor</t>
         </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M55" t="n">
+        <v>2024</v>
       </c>
     </row>
     <row r="56">
@@ -2905,6 +3349,14 @@
         <is>
           <t>Growth Funded by Debt</t>
         </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="M56" t="n">
+        <v>2024</v>
       </c>
     </row>
     <row r="57">
@@ -2947,6 +3399,14 @@
           <t>Growth Funded by Debt</t>
         </is>
       </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="M57" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2990,6 +3450,14 @@
           <t>Growth Funded by Debt</t>
         </is>
       </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="M58" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3033,6 +3501,14 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M59" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3077,6 +3553,14 @@
         <is>
           <t>Reinvestor</t>
         </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M60" t="n">
+        <v>2024</v>
       </c>
     </row>
     <row r="61">
@@ -3121,6 +3605,14 @@
           <t>Growth Funded by Debt</t>
         </is>
       </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="M61" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3166,6 +3658,14 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M62" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3211,6 +3711,14 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M63" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3256,6 +3764,14 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M64" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3301,6 +3817,14 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M65" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3346,6 +3870,14 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M66" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3391,6 +3923,14 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M67" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3435,6 +3975,14 @@
         <is>
           <t>Shareholder Returns</t>
         </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M68" t="n">
+        <v>2024</v>
       </c>
     </row>
     <row r="69">
@@ -3479,6 +4027,14 @@
           <t>Mixed</t>
         </is>
       </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="M69" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3523,6 +4079,14 @@
         <is>
           <t>Shareholder Returns</t>
         </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M70" t="n">
+        <v>2024</v>
       </c>
     </row>
     <row r="71">
@@ -3567,6 +4131,14 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M71" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3610,6 +4182,14 @@
           <t>Distress Signal</t>
         </is>
       </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
+      <c r="M72" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3653,6 +4233,14 @@
           <t>Growth Funded by Debt</t>
         </is>
       </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="M73" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3696,6 +4284,14 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M74" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3740,6 +4336,14 @@
         <is>
           <t>Shareholder Returns</t>
         </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M75" t="n">
+        <v>2024</v>
       </c>
     </row>
     <row r="76">
@@ -3784,6 +4388,14 @@
           <t>Liquidating Assets</t>
         </is>
       </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="M76" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3829,6 +4441,14 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M77" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3874,6 +4494,14 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M78" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3919,6 +4547,14 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M79" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3964,6 +4600,14 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M80" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4009,6 +4653,14 @@
           <t>Liquidating Assets</t>
         </is>
       </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="M81" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4053,6 +4705,14 @@
         <is>
           <t>Shareholder Returns</t>
         </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M82" t="n">
+        <v>2024</v>
       </c>
     </row>
     <row r="83">
@@ -4097,6 +4757,14 @@
           <t>Mixed</t>
         </is>
       </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="M83" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4142,6 +4810,14 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M84" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4187,6 +4863,14 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M85" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4231,6 +4915,14 @@
         <is>
           <t>Shareholder Returns</t>
         </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M86" t="n">
+        <v>2024</v>
       </c>
     </row>
     <row r="87">
@@ -4275,6 +4967,14 @@
           <t>Mixed</t>
         </is>
       </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="M87" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4318,6 +5018,14 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M88" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4363,6 +5071,14 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M89" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4407,6 +5123,14 @@
         <is>
           <t>Shareholder Returns</t>
         </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M90" t="n">
+        <v>2024</v>
       </c>
     </row>
     <row r="91">
@@ -4451,6 +5175,14 @@
           <t>Reinvestor</t>
         </is>
       </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="M91" t="n">
+        <v>2024</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4495,6 +5227,14 @@
         <is>
           <t>Mixed</t>
         </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="M92" t="n">
+        <v>2024</v>
       </c>
     </row>
     <row r="93">
@@ -4538,6 +5278,14 @@
         <is>
           <t>Mixed</t>
         </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="M93" t="n">
+        <v>2024</v>
       </c>
     </row>
   </sheetData>
@@ -4659,4 +5407,620 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>pattern_label</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>company_count</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>56</v>
+      </c>
+      <c r="C2" t="n">
+        <v>60.86956521739131</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C4" t="n">
+        <v>7.608695652173914</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1.08695652173913</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>12</v>
+      </c>
+      <c r="C6" t="n">
+        <v>13.04347826086956</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Cash Accumulator</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Pre-Revenue</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1.08695652173913</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>15</v>
+      </c>
+      <c r="C9" t="n">
+        <v>16.30434782608696</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>previous_pattern</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>current_pattern</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>company_count</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Pre-Revenue</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Pre-Revenue</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Pre-Revenue</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Pre-Revenue</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Cash Accumulator</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Pre-Revenue</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Pre-Revenue</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Pre-Revenue</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Cash Accumulator</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Cash Accumulator</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Cash Accumulator</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Cash Accumulator</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>